<commit_message>
fixing som2024 population groups names
</commit_message>
<xml_diff>
--- a/pin2024_cat/SOM_PIN2024.xlsx
+++ b/pin2024_cat/SOM_PIN2024.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted.sharepoint.com/sites/IMPACTHQ-PublicServices-IMPACT-Education/Documents partages/IMPACT - Education/Education - shared folder/PiN/PiN methodology studies 2025/new_dataset_testing/pin2024_cat/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acted-my.sharepoint.com/personal/martina_vit_impact-initiatives_org/Documents/PiN_app_dev/pin2024_cat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_17BDCEE3289B1917203650BF76E02B56DA514C28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C3F77E-7C92-46CF-A0F6-E3FE662A74D2}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_17BDCEE3289B1917203650BF76E02B56DA514C28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0786615-6CBE-4759-83BC-CA3A1A821E42}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="host" sheetId="1" r:id="rId1"/>
-    <sheet name="idp" sheetId="2" r:id="rId2"/>
+    <sheet name="affected_pop" sheetId="1" r:id="rId1"/>
+    <sheet name="recent_idp" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -2347,25 +2347,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C9824523CAB29F4DA646F20BAFE41B4C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c972c102b01d47663811fb2ebdbd1e4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5940141-1bc9-4c17-b1bc-e50f6b2083d6" xmlns:ns3="14cbb838-50ff-4dab-9c3f-cddf75f03c13" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bd0e8b72e466adcc572d3af37c1ebe05" ns2:_="" ns3:_="">
     <xsd:import namespace="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
@@ -2588,12 +2569,40 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5940141-1bc9-4c17-b1bc-e50f6b2083d6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4779FBD7-BA20-4C78-9B9B-D254683ED8B0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E8C48C8-8941-4238-B7BC-BA492FEB8FAE}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+    <ds:schemaRef ds:uri="14cbb838-50ff-4dab-9c3f-cddf75f03c13"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2607,5 +2616,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E8C48C8-8941-4238-B7BC-BA492FEB8FAE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4779FBD7-BA20-4C78-9B9B-D254683ED8B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b5940141-1bc9-4c17-b1bc-e50f6b2083d6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>